<commit_message>
Change the short ch TH to 0.8 as in the freeplay. Didn't change the 9 m sample, but did change 18m. Therefore, I ran the entire pipeline again for 18m
</commit_message>
<xml_diff>
--- a/Best ch pipeline/improved_best_channels_stat_18m_hammer.xlsx
+++ b/Best ch pipeline/improved_best_channels_stat_18m_hammer.xlsx
@@ -1287,7 +1287,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ch_1</t>
+          <t>ch_0</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1297,19 +1297,19 @@
         <v>30169</v>
       </c>
       <c r="H18" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J18" t="n">
-        <v>1043.241196979758</v>
+        <v>994.343080184657</v>
       </c>
       <c r="K18" t="n">
-        <v>879.4848484848485</v>
+        <v>806.1944444444445</v>
       </c>
       <c r="L18" t="n">
-        <v>517</v>
+        <v>460</v>
       </c>
     </row>
     <row r="19">

</xml_diff>